<commit_message>
CFTR nihai şampiyon düzeltmesi (RF/original) + nihai_sampiyonlar/SUREC/paket güncellendi
</commit_message>
<xml_diff>
--- a/SRC/Result/nihai_sampiyonlar.xlsx
+++ b/SRC/Result/nihai_sampiyonlar.xlsx
@@ -513,17 +513,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>dengeli-clustering (gercek benign ~1:1)</t>
+          <t>original</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>feature_selection</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>OOF-tuned</t>
+          <t>0.88</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -545,16 +545,16 @@
         <v>0.926</v>
       </c>
       <c r="L2" t="n">
-        <v>0.897</v>
+        <v>0.916</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Sinif-dengeli clustering (patojenik yanliligi giderildi)</t>
+          <t>(matris en iyisi; dengeli-clustering denendi ama gecemedi)</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Sartname F1 en yuksek + CM dengeli (FP3/FN0) + leak-free gercek benign</t>
+          <t>En yuksek F1 + guclu cv_auc (0.916) + recall 1.0 (FN=0). Saf cv_auc lideri CatBoost/clustering (0.994) alternatif</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Augmentasyon yaramadi; tek lever esik. Klinik: hic patojenik kacirmama onceligi</t>
+          <t>Augmentasyon yaramadi; tek lever esik. Klinik: hic patojenik kacirmama. Yuksek esikte F1 0.500</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CFTR nihai = CatBoost/clustering (AUC-tutarli secim, RF/F1 istisnasi kaldirildi) + birlesik AUC-vs-nihai tablosu + nihai_sampiyonlar ROC_AUC duzeltmesi
</commit_message>
<xml_diff>
--- a/SRC/Result/nihai_sampiyonlar.xlsx
+++ b/SRC/Result/nihai_sampiyonlar.xlsx
@@ -508,53 +508,51 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>original</t>
+          <t>clustering</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>feature_selection</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0.88</t>
-        </is>
+          <t>feature_subsample</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0.9</v>
       </c>
       <c r="F2" t="n">
-        <v>0.88</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="G2" t="n">
-        <v>0.756</v>
+        <v>0.612</v>
       </c>
       <c r="H2" t="n">
-        <v>0.861</v>
+        <v>0.76</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
       </c>
       <c r="J2" t="n">
-        <v>0.786</v>
+        <v>0.6879999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>0.926</v>
+        <v>0.9256</v>
       </c>
       <c r="L2" t="n">
-        <v>0.916</v>
+        <v>0.994</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>(matris en iyisi; dengeli-clustering denendi ama gecemedi)</t>
+          <t>(saf cv_auc lideri; AUC-tutarli secim)</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>En yuksek F1 + guclu cv_auc (0.916) + recall 1.0 (FN=0). Saf cv_auc lideri CatBoost/clustering (0.994) alternatif</t>
+          <t>Tum panellerle tutarli: sizintisiz cv_auc lideri (0.994). RF/original F1 daha yuksekti (0.880) ama cv_auc dusuk (0.916) -&gt; kucuk-test F1 iyimserligi; AUC-tutarlilik tercih edildi.</t>
         </is>
       </c>
     </row>

</xml_diff>